<commit_message>
Final submission: peer confirmations, fixed covers, defect log and walkthrough video
</commit_message>
<xml_diff>
--- a/Capstone_Project/06_Testing_Results_and_Evaluation/Group-3_Defect_Log.xlsx
+++ b/Capstone_Project/06_Testing_Results_and_Evaluation/Group-3_Defect_Log.xlsx
@@ -492,7 +492,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -661,7 +660,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Map startTime and endTime to start and end in loadSlots in BookSlot.jsx. Fix is in the working copy and not yet committed</t>
+          <t>Map startTime and endTime to start and end in loadSlots in BookSlot.jsx. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -721,7 +720,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Use /api/slots/mine and send startTime and endTime and map them when listing in LecturerSlots.jsx. Fix is in the working copy and not yet committed</t>
+          <t>Use /api/slots/mine and send startTime and endTime and map them when listing in LecturerSlots.jsx. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -731,7 +730,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>TC-25 and TC-33 and D-03_fix_LecturerSlots.patch</t>
+          <t>TC-25 and TC-33 and commit 09effbe</t>
         </is>
       </c>
     </row>
@@ -781,7 +780,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Added a Change time button on My bookings that lists the other open times of that lecturer and calls PATCH /api/bookings/:id/change. The bookings API now also returns lecturerId. Not yet committed</t>
+          <t>Added a Change time button on My bookings that lists the other open times of that lecturer and calls PATCH /api/bookings/:id/change. The bookings API now also returns lecturerId. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -841,7 +840,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Response interceptor in api.js clears the saved login and goes to /login with the message Your session has ended on a 401. Not yet committed</t>
+          <t>Response interceptor in api.js clears the saved login and goes to /login with the message Your session has ended on a 401. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -901,7 +900,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Login allows 10 wrong passwords per account and address in 15 minutes and then answers 429. Not yet committed</t>
+          <t>Login allows 10 wrong passwords per account and address in 15 minutes and then answers 429. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1021,7 +1020,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>The confirm step stays visible after an error unless the slot was taken. Not yet committed</t>
+          <t>The confirm step stays visible after an error unless the slot was taken. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1081,7 +1080,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Added an Edit button that fills the form and saves with PUT /api/slots/:id. Not yet committed</t>
+          <t>Added an Edit button that fills the form and saves with PUT /api/slots/:id. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1141,7 +1140,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>ProtectedRoute sends the user to their own home page. Not yet committed</t>
+          <t>ProtectedRoute sends the user to their own home page. Committed in 09effbe on 26 October 2026</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">

</xml_diff>